<commit_message>
WE HAVE A WINNER!
used the latest 'stable' model and added feed in L in master table
</commit_message>
<xml_diff>
--- a/data/Test Experiment/Test-MasterDataTable.xlsx
+++ b/data/Test Experiment/Test-MasterDataTable.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mydrive.gsk.com/personal/zach_a_hatzenbeller_gsk_com/Documents/Documents/GitHub/state-space-model/data/Test Experiment/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yl604392\Git\state-space-model\data\Test Experiment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3149" documentId="14_{29998BAB-B97E-4D42-B36C-5857DA37A7C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5292F756-0A1A-4558-84B1-7779BA5CD0CE}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED1254C4-4D75-4A8F-AEE2-0F1B38868770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-30" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MasterDataTable" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="4" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">MasterDataTable!$A$2:$AI$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">MasterDataTable!$A$2:$AJ$92</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="52">
   <si>
     <t>Batch Data</t>
   </si>
@@ -193,6 +193,9 @@
   </si>
   <si>
     <t>Volume from Reactor (L)</t>
+  </si>
+  <si>
+    <t>Daily Feed Amount (L)</t>
   </si>
 </sst>
 </file>
@@ -946,10 +949,10 @@
     <xf numFmtId="0" fontId="19" fillId="34" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="34" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="34" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="34" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="34" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
@@ -1314,25 +1317,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:AI92"/>
-  <sheetFormatPr defaultColWidth="14.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:AJ92"/>
+  <sheetFormatPr defaultColWidth="14.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.44140625" customWidth="1"/>
-    <col min="5" max="5" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="16" width="12.6640625" customWidth="1"/>
-    <col min="17" max="17" width="15.109375" customWidth="1"/>
-    <col min="18" max="18" width="16.109375" customWidth="1"/>
-    <col min="19" max="30" width="12.6640625" customWidth="1"/>
-    <col min="31" max="31" width="12.5546875" customWidth="1"/>
-    <col min="32" max="33" width="14.88671875" customWidth="1"/>
-    <col min="34" max="35" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="16" width="12.7109375" customWidth="1"/>
+    <col min="17" max="17" width="15.140625" customWidth="1"/>
+    <col min="18" max="18" width="16.140625" customWidth="1"/>
+    <col min="19" max="31" width="12.7109375" customWidth="1"/>
+    <col min="32" max="32" width="12.5703125" customWidth="1"/>
+    <col min="33" max="34" width="14.85546875" customWidth="1"/>
+    <col min="35" max="36" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:36" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
@@ -1368,16 +1371,17 @@
       <c r="AC1" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="AD1" s="31"/>
+      <c r="AD1" s="30"/>
       <c r="AE1" s="30"/>
-      <c r="AF1" s="26" t="s">
+      <c r="AF1" s="31"/>
+      <c r="AG1" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="AG1" s="27"/>
       <c r="AH1" s="27"/>
-      <c r="AI1" s="28"/>
-    </row>
-    <row r="2" spans="1:35" ht="30.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="AI1" s="27"/>
+      <c r="AJ1" s="28"/>
+    </row>
+    <row r="2" spans="1:36" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>4</v>
       </c>
@@ -1465,26 +1469,29 @@
       <c r="AC2" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="AD2" s="6" t="s">
+      <c r="AD2" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="AE2" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="AE2" s="6" t="s">
+      <c r="AF2" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="AF2" s="7" t="s">
+      <c r="AG2" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="AG2" s="15" t="s">
+      <c r="AH2" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="AH2" s="15" t="s">
+      <c r="AI2" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="AI2" s="6" t="s">
+      <c r="AJ2" s="6" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>36</v>
       </c>
@@ -1571,25 +1578,29 @@
         <v>0</v>
       </c>
       <c r="AD3" s="3">
+        <f>AC3/1000</f>
+        <v>0</v>
+      </c>
+      <c r="AE3" s="3">
         <v>0.18721000000000002</v>
       </c>
-      <c r="AE3" s="13">
+      <c r="AF3" s="13">
         <v>187.21</v>
       </c>
-      <c r="AF3" s="2">
+      <c r="AG3" s="2">
         <v>190</v>
       </c>
-      <c r="AG3" s="3">
+      <c r="AH3" s="3">
         <v>35</v>
       </c>
-      <c r="AH3" s="3">
+      <c r="AI3" s="3">
         <v>6.75</v>
       </c>
-      <c r="AI3" s="13">
+      <c r="AJ3" s="13">
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>37</v>
       </c>
@@ -1672,25 +1683,29 @@
         <v>0</v>
       </c>
       <c r="AD4" s="32">
+        <f t="shared" ref="AD4:AD67" si="0">AC4/1000</f>
+        <v>0</v>
+      </c>
+      <c r="AE4">
         <v>0.18721000000000002</v>
       </c>
-      <c r="AE4" s="12">
+      <c r="AF4" s="12">
         <v>187.21</v>
       </c>
-      <c r="AF4" s="1">
+      <c r="AG4" s="1">
         <v>190</v>
       </c>
-      <c r="AG4">
+      <c r="AH4">
         <v>35</v>
       </c>
-      <c r="AH4">
+      <c r="AI4">
         <v>7.45</v>
       </c>
-      <c r="AI4" s="12">
+      <c r="AJ4" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>38</v>
       </c>
@@ -1779,25 +1794,29 @@
         <v>0</v>
       </c>
       <c r="AD5" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE5">
         <v>0.18624000000000002</v>
       </c>
-      <c r="AE5" s="12">
+      <c r="AF5" s="12">
         <v>186.24</v>
       </c>
-      <c r="AF5" s="1">
+      <c r="AG5" s="1">
         <v>190</v>
       </c>
-      <c r="AG5">
+      <c r="AH5">
         <v>38</v>
       </c>
-      <c r="AH5">
+      <c r="AI5">
         <v>6.75</v>
       </c>
-      <c r="AI5" s="12">
+      <c r="AJ5" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>39</v>
       </c>
@@ -1883,25 +1902,29 @@
         <v>0</v>
       </c>
       <c r="AD6" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE6">
         <v>0.18721000000000002</v>
       </c>
-      <c r="AE6" s="12">
+      <c r="AF6" s="12">
         <v>187.21</v>
       </c>
-      <c r="AF6" s="1">
+      <c r="AG6" s="1">
         <v>190</v>
       </c>
-      <c r="AG6">
+      <c r="AH6">
         <v>36.5</v>
       </c>
-      <c r="AH6">
+      <c r="AI6">
         <v>7.1</v>
       </c>
-      <c r="AI6" s="12">
+      <c r="AJ6" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>40</v>
       </c>
@@ -1990,25 +2013,29 @@
         <v>0</v>
       </c>
       <c r="AD7" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE7">
         <v>0.18624000000000002</v>
       </c>
-      <c r="AE7" s="12">
+      <c r="AF7" s="12">
         <v>186.24</v>
       </c>
-      <c r="AF7" s="1">
+      <c r="AG7" s="1">
         <v>190</v>
       </c>
-      <c r="AG7">
+      <c r="AH7">
         <v>36.5</v>
       </c>
-      <c r="AH7">
+      <c r="AI7">
         <v>7.1</v>
       </c>
-      <c r="AI7" s="12">
+      <c r="AJ7" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:36" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>41</v>
       </c>
@@ -2097,25 +2124,29 @@
         <v>0</v>
       </c>
       <c r="AD8" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE8" s="5">
         <v>0.18721000000000002</v>
       </c>
-      <c r="AE8" s="14">
+      <c r="AF8" s="14">
         <v>187.21</v>
       </c>
-      <c r="AF8" s="4">
+      <c r="AG8" s="4">
         <v>190</v>
       </c>
-      <c r="AG8" s="5">
+      <c r="AH8" s="5">
         <v>35</v>
       </c>
-      <c r="AH8" s="5">
+      <c r="AI8" s="5">
         <v>7.45</v>
       </c>
-      <c r="AI8" s="14">
+      <c r="AJ8" s="14">
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>36</v>
       </c>
@@ -2202,25 +2233,29 @@
         <v>0</v>
       </c>
       <c r="AD9" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE9" s="3">
         <v>0.18618000000000001</v>
       </c>
-      <c r="AE9" s="13">
+      <c r="AF9" s="13">
         <v>186.18</v>
       </c>
-      <c r="AF9" s="2">
+      <c r="AG9" s="2">
         <v>190</v>
       </c>
-      <c r="AG9" s="3">
+      <c r="AH9" s="3">
         <v>35</v>
       </c>
-      <c r="AH9" s="3">
+      <c r="AI9" s="3">
         <v>6.75</v>
       </c>
-      <c r="AI9" s="13">
+      <c r="AJ9" s="13">
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>37</v>
       </c>
@@ -2306,25 +2341,29 @@
         <v>0</v>
       </c>
       <c r="AD10" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE10">
         <v>0.18619999999999998</v>
       </c>
-      <c r="AE10" s="12">
+      <c r="AF10" s="12">
         <v>186.2</v>
       </c>
-      <c r="AF10" s="1">
+      <c r="AG10" s="1">
         <v>190</v>
       </c>
-      <c r="AG10">
+      <c r="AH10">
         <v>35</v>
       </c>
-      <c r="AH10">
+      <c r="AI10">
         <v>7.45</v>
       </c>
-      <c r="AI10" s="12">
+      <c r="AJ10" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>38</v>
       </c>
@@ -2410,25 +2449,29 @@
         <v>0</v>
       </c>
       <c r="AD11" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE11">
         <v>0.18340999999999999</v>
       </c>
-      <c r="AE11" s="12">
+      <c r="AF11" s="12">
         <v>183.41</v>
       </c>
-      <c r="AF11" s="1">
+      <c r="AG11" s="1">
         <v>190</v>
       </c>
-      <c r="AG11">
+      <c r="AH11">
         <v>38</v>
       </c>
-      <c r="AH11">
+      <c r="AI11">
         <v>6.75</v>
       </c>
-      <c r="AI11" s="12">
+      <c r="AJ11" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>39</v>
       </c>
@@ -2514,25 +2557,29 @@
         <v>0</v>
       </c>
       <c r="AD12" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE12">
         <v>0.18439</v>
       </c>
-      <c r="AE12" s="12">
+      <c r="AF12" s="12">
         <v>184.39</v>
       </c>
-      <c r="AF12" s="1">
+      <c r="AG12" s="1">
         <v>190</v>
       </c>
-      <c r="AG12">
+      <c r="AH12">
         <v>36.5</v>
       </c>
-      <c r="AH12">
+      <c r="AI12">
         <v>7.1</v>
       </c>
-      <c r="AI12" s="12">
+      <c r="AJ12" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>40</v>
       </c>
@@ -2621,25 +2668,29 @@
         <v>0</v>
       </c>
       <c r="AD13" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE13">
         <v>0.18342</v>
       </c>
-      <c r="AE13" s="12">
+      <c r="AF13" s="12">
         <v>183.42</v>
       </c>
-      <c r="AF13" s="1">
+      <c r="AG13" s="1">
         <v>190</v>
       </c>
-      <c r="AG13">
+      <c r="AH13">
         <v>36.5</v>
       </c>
-      <c r="AH13">
+      <c r="AI13">
         <v>7.1</v>
       </c>
-      <c r="AI13" s="12">
+      <c r="AJ13" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>41</v>
       </c>
@@ -2728,25 +2779,29 @@
         <v>0</v>
       </c>
       <c r="AD14" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE14" s="5">
         <v>0.18440000000000001</v>
       </c>
-      <c r="AE14" s="14">
+      <c r="AF14" s="14">
         <v>184.4</v>
       </c>
-      <c r="AF14" s="4">
+      <c r="AG14" s="4">
         <v>190</v>
       </c>
-      <c r="AG14" s="5">
+      <c r="AH14" s="5">
         <v>35</v>
       </c>
-      <c r="AH14" s="5">
+      <c r="AI14" s="5">
         <v>7.45</v>
       </c>
-      <c r="AI14" s="14">
+      <c r="AJ14" s="14">
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>36</v>
       </c>
@@ -2835,25 +2890,29 @@
         <v>0</v>
       </c>
       <c r="AD15" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE15">
         <v>0.18155000000000002</v>
       </c>
-      <c r="AE15" s="12">
+      <c r="AF15" s="12">
         <v>181.55</v>
       </c>
-      <c r="AF15" s="1">
+      <c r="AG15" s="1">
         <v>190</v>
       </c>
-      <c r="AG15">
+      <c r="AH15">
         <v>35</v>
       </c>
-      <c r="AH15">
+      <c r="AI15">
         <v>6.75</v>
       </c>
-      <c r="AI15" s="12">
+      <c r="AJ15" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>37</v>
       </c>
@@ -2942,25 +3001,29 @@
         <v>0</v>
       </c>
       <c r="AD16" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE16">
         <v>0.18158000000000002</v>
       </c>
-      <c r="AE16" s="12">
+      <c r="AF16" s="12">
         <v>181.58</v>
       </c>
-      <c r="AF16" s="1">
+      <c r="AG16" s="1">
         <v>190</v>
       </c>
-      <c r="AG16">
+      <c r="AH16">
         <v>35</v>
       </c>
-      <c r="AH16">
+      <c r="AI16">
         <v>7.45</v>
       </c>
-      <c r="AI16" s="12">
+      <c r="AJ16" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>38</v>
       </c>
@@ -3049,25 +3112,29 @@
         <v>0</v>
       </c>
       <c r="AD17" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE17">
         <v>0.18058000000000002</v>
       </c>
-      <c r="AE17" s="12">
+      <c r="AF17" s="12">
         <v>180.58</v>
       </c>
-      <c r="AF17" s="1">
+      <c r="AG17" s="1">
         <v>190</v>
       </c>
-      <c r="AG17">
+      <c r="AH17">
         <v>38</v>
       </c>
-      <c r="AH17">
+      <c r="AI17">
         <v>6.75</v>
       </c>
-      <c r="AI17" s="12">
+      <c r="AJ17" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>39</v>
       </c>
@@ -3156,25 +3223,29 @@
         <v>0</v>
       </c>
       <c r="AD18" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE18">
         <v>0.18156999999999998</v>
       </c>
-      <c r="AE18" s="12">
+      <c r="AF18" s="12">
         <v>181.57</v>
       </c>
-      <c r="AF18" s="1">
+      <c r="AG18" s="1">
         <v>190</v>
       </c>
-      <c r="AG18">
+      <c r="AH18">
         <v>36.5</v>
       </c>
-      <c r="AH18">
+      <c r="AI18">
         <v>7.1</v>
       </c>
-      <c r="AI18" s="12">
+      <c r="AJ18" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>40</v>
       </c>
@@ -3263,25 +3334,29 @@
         <v>0</v>
       </c>
       <c r="AD19" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE19">
         <v>0.18059</v>
       </c>
-      <c r="AE19" s="12">
+      <c r="AF19" s="12">
         <v>180.59</v>
       </c>
-      <c r="AF19" s="1">
+      <c r="AG19" s="1">
         <v>190</v>
       </c>
-      <c r="AG19">
+      <c r="AH19">
         <v>36.5</v>
       </c>
-      <c r="AH19">
+      <c r="AI19">
         <v>7.1</v>
       </c>
-      <c r="AI19" s="12">
+      <c r="AJ19" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="20" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:36" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>41</v>
       </c>
@@ -3370,25 +3445,29 @@
         <v>0</v>
       </c>
       <c r="AD20" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE20">
         <v>0.18158000000000002</v>
       </c>
-      <c r="AE20" s="12">
+      <c r="AF20" s="12">
         <v>181.58</v>
       </c>
-      <c r="AF20" s="1">
+      <c r="AG20" s="1">
         <v>190</v>
       </c>
-      <c r="AG20">
+      <c r="AH20">
         <v>35</v>
       </c>
-      <c r="AH20">
+      <c r="AI20">
         <v>7.45</v>
       </c>
-      <c r="AI20" s="12">
+      <c r="AJ20" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>36</v>
       </c>
@@ -3477,25 +3556,29 @@
         <v>0</v>
       </c>
       <c r="AD21" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE21" s="3">
         <v>0.18052000000000001</v>
       </c>
-      <c r="AE21" s="13">
+      <c r="AF21" s="13">
         <v>180.52</v>
       </c>
-      <c r="AF21" s="2">
+      <c r="AG21" s="2">
         <v>190</v>
       </c>
-      <c r="AG21" s="3">
+      <c r="AH21" s="3">
         <v>35</v>
       </c>
-      <c r="AH21" s="3">
+      <c r="AI21" s="3">
         <v>6.75</v>
       </c>
-      <c r="AI21" s="13">
+      <c r="AJ21" s="13">
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>37</v>
       </c>
@@ -3584,25 +3667,29 @@
         <v>0</v>
       </c>
       <c r="AD22" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE22">
         <v>0.18056</v>
       </c>
-      <c r="AE22" s="12">
+      <c r="AF22" s="12">
         <v>180.56</v>
       </c>
-      <c r="AF22" s="1">
+      <c r="AG22" s="1">
         <v>190</v>
       </c>
-      <c r="AG22">
+      <c r="AH22">
         <v>35</v>
       </c>
-      <c r="AH22">
+      <c r="AI22">
         <v>7.45</v>
       </c>
-      <c r="AI22" s="12">
+      <c r="AJ22" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>38</v>
       </c>
@@ -3691,25 +3778,29 @@
         <v>0</v>
       </c>
       <c r="AD23" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE23">
         <v>0.17954000000000001</v>
       </c>
-      <c r="AE23" s="12">
+      <c r="AF23" s="12">
         <v>179.54</v>
       </c>
-      <c r="AF23" s="1">
+      <c r="AG23" s="1">
         <v>190</v>
       </c>
-      <c r="AG23">
+      <c r="AH23">
         <v>38</v>
       </c>
-      <c r="AH23">
+      <c r="AI23">
         <v>6.75</v>
       </c>
-      <c r="AI23" s="12">
+      <c r="AJ23" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="24" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>39</v>
       </c>
@@ -3798,25 +3889,29 @@
         <v>0</v>
       </c>
       <c r="AD24" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE24">
         <v>0.18055000000000002</v>
       </c>
-      <c r="AE24" s="12">
+      <c r="AF24" s="12">
         <v>180.55</v>
       </c>
-      <c r="AF24" s="1">
+      <c r="AG24" s="1">
         <v>190</v>
       </c>
-      <c r="AG24">
+      <c r="AH24">
         <v>36.5</v>
       </c>
-      <c r="AH24">
+      <c r="AI24">
         <v>7.1</v>
       </c>
-      <c r="AI24" s="12">
+      <c r="AJ24" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="25" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>40</v>
       </c>
@@ -3905,25 +4000,29 @@
         <v>0</v>
       </c>
       <c r="AD25" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE25">
         <v>0.17956999999999998</v>
       </c>
-      <c r="AE25" s="12">
+      <c r="AF25" s="12">
         <v>179.57</v>
       </c>
-      <c r="AF25" s="1">
+      <c r="AG25" s="1">
         <v>190</v>
       </c>
-      <c r="AG25">
+      <c r="AH25">
         <v>36.5</v>
       </c>
-      <c r="AH25">
+      <c r="AI25">
         <v>7.1</v>
       </c>
-      <c r="AI25" s="12">
+      <c r="AJ25" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="26" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:36" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>41</v>
       </c>
@@ -4012,25 +4111,29 @@
         <v>0</v>
       </c>
       <c r="AD26" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE26" s="5">
         <v>0.18056</v>
       </c>
-      <c r="AE26" s="14">
+      <c r="AF26" s="14">
         <v>180.56</v>
       </c>
-      <c r="AF26" s="4">
+      <c r="AG26" s="4">
         <v>190</v>
       </c>
-      <c r="AG26" s="5">
+      <c r="AH26" s="5">
         <v>35</v>
       </c>
-      <c r="AH26" s="5">
+      <c r="AI26" s="5">
         <v>7.45</v>
       </c>
-      <c r="AI26" s="14">
+      <c r="AJ26" s="14">
         <v>40</v>
       </c>
     </row>
-    <row r="27" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>36</v>
       </c>
@@ -4119,25 +4222,29 @@
         <v>7.6</v>
       </c>
       <c r="AD27" s="32">
+        <f t="shared" si="0"/>
+        <v>7.6E-3</v>
+      </c>
+      <c r="AE27">
         <v>0.1835</v>
       </c>
-      <c r="AE27" s="12">
+      <c r="AF27" s="12">
         <v>183.5</v>
       </c>
-      <c r="AF27" s="1">
+      <c r="AG27" s="1">
         <v>190</v>
       </c>
-      <c r="AG27">
+      <c r="AH27">
         <v>35</v>
       </c>
-      <c r="AH27">
+      <c r="AI27">
         <v>6.75</v>
       </c>
-      <c r="AI27" s="12">
+      <c r="AJ27" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="28" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>37</v>
       </c>
@@ -4226,25 +4333,29 @@
         <v>11.4</v>
       </c>
       <c r="AD28" s="32">
+        <f t="shared" si="0"/>
+        <v>1.14E-2</v>
+      </c>
+      <c r="AE28">
         <v>0.17596000000000001</v>
       </c>
-      <c r="AE28" s="12">
+      <c r="AF28" s="12">
         <v>175.96</v>
       </c>
-      <c r="AF28" s="1">
+      <c r="AG28" s="1">
         <v>190</v>
       </c>
-      <c r="AG28">
+      <c r="AH28">
         <v>35</v>
       </c>
-      <c r="AH28">
+      <c r="AI28">
         <v>7.45</v>
       </c>
-      <c r="AI28" s="12">
+      <c r="AJ28" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="29" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>38</v>
       </c>
@@ -4333,25 +4444,29 @@
         <v>11.4</v>
       </c>
       <c r="AD29" s="32">
+        <f t="shared" si="0"/>
+        <v>1.14E-2</v>
+      </c>
+      <c r="AE29">
         <v>0.18633000000000002</v>
       </c>
-      <c r="AE29" s="12">
+      <c r="AF29" s="12">
         <v>186.33</v>
       </c>
-      <c r="AF29" s="1">
+      <c r="AG29" s="1">
         <v>190</v>
       </c>
-      <c r="AG29">
+      <c r="AH29">
         <v>38</v>
       </c>
-      <c r="AH29">
+      <c r="AI29">
         <v>6.75</v>
       </c>
-      <c r="AI29" s="12">
+      <c r="AJ29" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="30" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>39</v>
       </c>
@@ -4440,25 +4555,29 @@
         <v>9.5</v>
       </c>
       <c r="AD30" s="32">
+        <f t="shared" si="0"/>
+        <v>9.4999999999999998E-3</v>
+      </c>
+      <c r="AE30">
         <v>0.17593999999999999</v>
       </c>
-      <c r="AE30" s="12">
+      <c r="AF30" s="12">
         <v>175.94</v>
       </c>
-      <c r="AF30" s="1">
+      <c r="AG30" s="1">
         <v>190</v>
       </c>
-      <c r="AG30">
+      <c r="AH30">
         <v>36.5</v>
       </c>
-      <c r="AH30">
+      <c r="AI30">
         <v>7.1</v>
       </c>
-      <c r="AI30" s="12">
+      <c r="AJ30" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="31" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>40</v>
       </c>
@@ -4547,25 +4666,29 @@
         <v>9.5</v>
       </c>
       <c r="AD31" s="32">
+        <f t="shared" si="0"/>
+        <v>9.4999999999999998E-3</v>
+      </c>
+      <c r="AE31">
         <v>0.17496999999999999</v>
       </c>
-      <c r="AE31" s="12">
+      <c r="AF31" s="12">
         <v>174.97</v>
       </c>
-      <c r="AF31" s="1">
+      <c r="AG31" s="1">
         <v>190</v>
       </c>
-      <c r="AG31">
+      <c r="AH31">
         <v>36.5</v>
       </c>
-      <c r="AH31">
+      <c r="AI31">
         <v>7.1</v>
       </c>
-      <c r="AI31" s="12">
+      <c r="AJ31" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="32" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:36" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>41</v>
       </c>
@@ -4654,25 +4777,29 @@
         <v>7.6</v>
       </c>
       <c r="AD32" s="32">
+        <f t="shared" si="0"/>
+        <v>7.6E-3</v>
+      </c>
+      <c r="AE32">
         <v>0.17595</v>
       </c>
-      <c r="AE32" s="12">
+      <c r="AF32" s="12">
         <v>175.95</v>
       </c>
-      <c r="AF32" s="1">
+      <c r="AG32" s="1">
         <v>190</v>
       </c>
-      <c r="AG32">
+      <c r="AH32">
         <v>35</v>
       </c>
-      <c r="AH32">
+      <c r="AI32">
         <v>7.45</v>
       </c>
-      <c r="AI32" s="12">
+      <c r="AJ32" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="33" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>36</v>
       </c>
@@ -4761,25 +4888,29 @@
         <v>0</v>
       </c>
       <c r="AD33" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE33" s="3">
         <v>0.18068999999999999</v>
       </c>
-      <c r="AE33" s="13">
+      <c r="AF33" s="13">
         <v>180.69</v>
       </c>
-      <c r="AF33" s="2">
+      <c r="AG33" s="2">
         <v>190</v>
       </c>
-      <c r="AG33" s="3">
+      <c r="AH33" s="3">
         <v>35</v>
       </c>
-      <c r="AH33" s="3">
+      <c r="AI33" s="3">
         <v>6.75</v>
       </c>
-      <c r="AI33" s="13">
+      <c r="AJ33" s="13">
         <v>40</v>
       </c>
     </row>
-    <row r="34" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>37</v>
       </c>
@@ -4868,25 +4999,29 @@
         <v>0</v>
       </c>
       <c r="AD34" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE34">
         <v>0.18506999999999998</v>
       </c>
-      <c r="AE34" s="12">
+      <c r="AF34" s="12">
         <v>185.07</v>
       </c>
-      <c r="AF34" s="1">
+      <c r="AG34" s="1">
         <v>190</v>
       </c>
-      <c r="AG34">
+      <c r="AH34">
         <v>35</v>
       </c>
-      <c r="AH34">
+      <c r="AI34">
         <v>7.45</v>
       </c>
-      <c r="AI34" s="12">
+      <c r="AJ34" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="35" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>38</v>
       </c>
@@ -4975,25 +5110,29 @@
         <v>0</v>
       </c>
       <c r="AD35" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE35">
         <v>0.18350999999999998</v>
       </c>
-      <c r="AE35" s="12">
+      <c r="AF35" s="12">
         <v>183.51</v>
       </c>
-      <c r="AF35" s="1">
+      <c r="AG35" s="1">
         <v>190</v>
       </c>
-      <c r="AG35">
+      <c r="AH35">
         <v>38</v>
       </c>
-      <c r="AH35">
+      <c r="AI35">
         <v>6.75</v>
       </c>
-      <c r="AI35" s="12">
+      <c r="AJ35" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="36" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>39</v>
       </c>
@@ -5082,25 +5221,29 @@
         <v>0</v>
       </c>
       <c r="AD36" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE36">
         <v>0.18264</v>
       </c>
-      <c r="AE36" s="12">
+      <c r="AF36" s="12">
         <v>182.64</v>
       </c>
-      <c r="AF36" s="1">
+      <c r="AG36" s="1">
         <v>190</v>
       </c>
-      <c r="AG36">
+      <c r="AH36">
         <v>36.5</v>
       </c>
-      <c r="AH36">
+      <c r="AI36">
         <v>7.1</v>
       </c>
-      <c r="AI36" s="12">
+      <c r="AJ36" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="37" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>40</v>
       </c>
@@ -5189,25 +5332,29 @@
         <v>0</v>
       </c>
       <c r="AD37" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE37">
         <v>0.18261000000000002</v>
       </c>
-      <c r="AE37" s="12">
+      <c r="AF37" s="12">
         <v>182.61</v>
       </c>
-      <c r="AF37" s="1">
+      <c r="AG37" s="1">
         <v>190</v>
       </c>
-      <c r="AG37">
+      <c r="AH37">
         <v>36.5</v>
       </c>
-      <c r="AH37">
+      <c r="AI37">
         <v>7.1</v>
       </c>
-      <c r="AI37" s="12">
+      <c r="AJ37" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="38" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:36" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>41</v>
       </c>
@@ -5296,25 +5443,29 @@
         <v>0</v>
       </c>
       <c r="AD38" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE38" s="5">
         <v>0.18250999999999998</v>
       </c>
-      <c r="AE38" s="14">
+      <c r="AF38" s="14">
         <v>182.51</v>
       </c>
-      <c r="AF38" s="4">
+      <c r="AG38" s="4">
         <v>190</v>
       </c>
-      <c r="AG38" s="5">
+      <c r="AH38" s="5">
         <v>35</v>
       </c>
-      <c r="AH38" s="5">
+      <c r="AI38" s="5">
         <v>7.45</v>
       </c>
-      <c r="AI38" s="14">
+      <c r="AJ38" s="14">
         <v>40</v>
       </c>
     </row>
-    <row r="39" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>36</v>
       </c>
@@ -5403,25 +5554,29 @@
         <v>7.6</v>
       </c>
       <c r="AD39" s="32">
+        <f t="shared" si="0"/>
+        <v>7.6E-3</v>
+      </c>
+      <c r="AE39">
         <v>0.18727000000000002</v>
       </c>
-      <c r="AE39" s="12">
+      <c r="AF39" s="12">
         <v>187.27</v>
       </c>
-      <c r="AF39" s="1">
+      <c r="AG39" s="1">
         <v>190</v>
       </c>
-      <c r="AG39">
+      <c r="AH39">
         <v>35</v>
       </c>
-      <c r="AH39">
+      <c r="AI39">
         <v>6.75</v>
       </c>
-      <c r="AI39" s="12">
+      <c r="AJ39" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="40" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>37</v>
       </c>
@@ -5510,25 +5665,29 @@
         <v>11.4</v>
       </c>
       <c r="AD40" s="32">
+        <f t="shared" si="0"/>
+        <v>1.14E-2</v>
+      </c>
+      <c r="AE40">
         <v>0.18627000000000002</v>
       </c>
-      <c r="AE40" s="12">
+      <c r="AF40" s="12">
         <v>186.27</v>
       </c>
-      <c r="AF40" s="1">
+      <c r="AG40" s="1">
         <v>190</v>
       </c>
-      <c r="AG40">
+      <c r="AH40">
         <v>35</v>
       </c>
-      <c r="AH40">
+      <c r="AI40">
         <v>7.45</v>
       </c>
-      <c r="AI40" s="12">
+      <c r="AJ40" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="41" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>38</v>
       </c>
@@ -5617,25 +5776,29 @@
         <v>11.4</v>
       </c>
       <c r="AD41" s="32">
+        <f t="shared" si="0"/>
+        <v>1.14E-2</v>
+      </c>
+      <c r="AE41">
         <v>0.19388</v>
       </c>
-      <c r="AE41" s="12">
+      <c r="AF41" s="12">
         <v>193.88</v>
       </c>
-      <c r="AF41" s="1">
+      <c r="AG41" s="1">
         <v>190</v>
       </c>
-      <c r="AG41">
+      <c r="AH41">
         <v>38</v>
       </c>
-      <c r="AH41">
+      <c r="AI41">
         <v>6.75</v>
       </c>
-      <c r="AI41" s="12">
+      <c r="AJ41" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>39</v>
       </c>
@@ -5724,25 +5887,29 @@
         <v>9.5</v>
       </c>
       <c r="AD42" s="32">
+        <f t="shared" si="0"/>
+        <v>9.4999999999999998E-3</v>
+      </c>
+      <c r="AE42">
         <v>0.18339</v>
       </c>
-      <c r="AE42" s="12">
+      <c r="AF42" s="12">
         <v>183.39</v>
       </c>
-      <c r="AF42" s="1">
+      <c r="AG42" s="1">
         <v>190</v>
       </c>
-      <c r="AG42">
+      <c r="AH42">
         <v>36.5</v>
       </c>
-      <c r="AH42">
+      <c r="AI42">
         <v>7.1</v>
       </c>
-      <c r="AI42" s="12">
+      <c r="AJ42" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>40</v>
       </c>
@@ -5831,25 +5998,29 @@
         <v>9.5</v>
       </c>
       <c r="AD43" s="32">
+        <f t="shared" si="0"/>
+        <v>9.4999999999999998E-3</v>
+      </c>
+      <c r="AE43">
         <v>0.18159999999999998</v>
       </c>
-      <c r="AE43" s="12">
+      <c r="AF43" s="12">
         <v>181.6</v>
       </c>
-      <c r="AF43" s="1">
+      <c r="AG43" s="1">
         <v>190</v>
       </c>
-      <c r="AG43">
+      <c r="AH43">
         <v>36.5</v>
       </c>
-      <c r="AH43">
+      <c r="AI43">
         <v>7.1</v>
       </c>
-      <c r="AI43" s="12">
+      <c r="AJ43" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="44" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:36" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>41</v>
       </c>
@@ -5938,25 +6109,29 @@
         <v>7.6</v>
       </c>
       <c r="AD44" s="32">
+        <f t="shared" si="0"/>
+        <v>7.6E-3</v>
+      </c>
+      <c r="AE44">
         <v>0.18395</v>
       </c>
-      <c r="AE44" s="12">
+      <c r="AF44" s="12">
         <v>183.95</v>
       </c>
-      <c r="AF44" s="1">
+      <c r="AG44" s="1">
         <v>190</v>
       </c>
-      <c r="AG44">
+      <c r="AH44">
         <v>35</v>
       </c>
-      <c r="AH44">
+      <c r="AI44">
         <v>7.45</v>
       </c>
-      <c r="AI44" s="12">
+      <c r="AJ44" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="45" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>36</v>
       </c>
@@ -6045,25 +6220,29 @@
         <v>0</v>
       </c>
       <c r="AD45" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE45" s="3">
         <v>0.18446000000000001</v>
       </c>
-      <c r="AE45" s="13">
+      <c r="AF45" s="13">
         <v>184.46</v>
       </c>
-      <c r="AF45" s="2">
+      <c r="AG45" s="2">
         <v>190</v>
       </c>
-      <c r="AG45" s="3">
+      <c r="AH45" s="3">
         <v>35</v>
       </c>
-      <c r="AH45" s="3">
+      <c r="AI45" s="3">
         <v>6.75</v>
       </c>
-      <c r="AI45" s="13">
+      <c r="AJ45" s="13">
         <v>40</v>
       </c>
     </row>
-    <row r="46" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>37</v>
       </c>
@@ -6152,25 +6331,29 @@
         <v>0</v>
       </c>
       <c r="AD46" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE46">
         <v>0.19763999999999998</v>
       </c>
-      <c r="AE46" s="12">
+      <c r="AF46" s="12">
         <v>197.64</v>
       </c>
-      <c r="AF46" s="1">
+      <c r="AG46" s="1">
         <v>190</v>
       </c>
-      <c r="AG46">
+      <c r="AH46">
         <v>35</v>
       </c>
-      <c r="AH46">
+      <c r="AI46">
         <v>7.45</v>
       </c>
-      <c r="AI46" s="12">
+      <c r="AJ46" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="47" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>38</v>
       </c>
@@ -6259,25 +6442,29 @@
         <v>0</v>
       </c>
       <c r="AD47" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE47">
         <v>0.19238</v>
       </c>
-      <c r="AE47" s="12">
+      <c r="AF47" s="12">
         <v>192.38</v>
       </c>
-      <c r="AF47" s="1">
+      <c r="AG47" s="1">
         <v>190</v>
       </c>
-      <c r="AG47">
+      <c r="AH47">
         <v>38</v>
       </c>
-      <c r="AH47">
+      <c r="AI47">
         <v>6.75</v>
       </c>
-      <c r="AI47" s="12">
+      <c r="AJ47" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="48" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>39</v>
       </c>
@@ -6366,25 +6553,29 @@
         <v>0</v>
       </c>
       <c r="AD48" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE48">
         <v>0.19024000000000002</v>
       </c>
-      <c r="AE48" s="12">
+      <c r="AF48" s="12">
         <v>190.24</v>
       </c>
-      <c r="AF48" s="1">
+      <c r="AG48" s="1">
         <v>190</v>
       </c>
-      <c r="AG48">
+      <c r="AH48">
         <v>36.5</v>
       </c>
-      <c r="AH48">
+      <c r="AI48">
         <v>7.1</v>
       </c>
-      <c r="AI48" s="12">
+      <c r="AJ48" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="49" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>40</v>
       </c>
@@ -6473,25 +6664,29 @@
         <v>0</v>
       </c>
       <c r="AD49" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE49">
         <v>0.19043000000000002</v>
       </c>
-      <c r="AE49" s="12">
+      <c r="AF49" s="12">
         <v>190.43</v>
       </c>
-      <c r="AF49" s="1">
+      <c r="AG49" s="1">
         <v>190</v>
       </c>
-      <c r="AG49">
+      <c r="AH49">
         <v>36.5</v>
       </c>
-      <c r="AH49">
+      <c r="AI49">
         <v>7.1</v>
       </c>
-      <c r="AI49" s="12">
+      <c r="AJ49" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="50" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:36" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
         <v>41</v>
       </c>
@@ -6580,25 +6775,29 @@
         <v>0</v>
       </c>
       <c r="AD50" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE50" s="5">
         <v>0.19122</v>
       </c>
-      <c r="AE50" s="14">
+      <c r="AF50" s="14">
         <v>191.22</v>
       </c>
-      <c r="AF50" s="4">
+      <c r="AG50" s="4">
         <v>190</v>
       </c>
-      <c r="AG50" s="5">
+      <c r="AH50" s="5">
         <v>35</v>
       </c>
-      <c r="AH50" s="5">
+      <c r="AI50" s="5">
         <v>7.45</v>
       </c>
-      <c r="AI50" s="14">
+      <c r="AJ50" s="14">
         <v>40</v>
       </c>
     </row>
-    <row r="51" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>36</v>
       </c>
@@ -6687,25 +6886,29 @@
         <v>7.6</v>
       </c>
       <c r="AD51" s="32">
+        <f t="shared" si="0"/>
+        <v>7.6E-3</v>
+      </c>
+      <c r="AE51">
         <v>0.18744</v>
       </c>
-      <c r="AE51" s="12">
+      <c r="AF51" s="12">
         <v>187.44</v>
       </c>
-      <c r="AF51" s="1">
+      <c r="AG51" s="1">
         <v>190</v>
       </c>
-      <c r="AG51">
+      <c r="AH51">
         <v>35</v>
       </c>
-      <c r="AH51">
+      <c r="AI51">
         <v>6.75</v>
       </c>
-      <c r="AI51" s="12">
+      <c r="AJ51" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="52" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>37</v>
       </c>
@@ -6794,25 +6997,29 @@
         <v>11.4</v>
       </c>
       <c r="AD52" s="32">
+        <f t="shared" si="0"/>
+        <v>1.14E-2</v>
+      </c>
+      <c r="AE52">
         <v>0.19797999999999999</v>
       </c>
-      <c r="AE52" s="12">
+      <c r="AF52" s="12">
         <v>197.98</v>
       </c>
-      <c r="AF52" s="1">
+      <c r="AG52" s="1">
         <v>190</v>
       </c>
-      <c r="AG52">
+      <c r="AH52">
         <v>35</v>
       </c>
-      <c r="AH52">
+      <c r="AI52">
         <v>7.45</v>
       </c>
-      <c r="AI52" s="12">
+      <c r="AJ52" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="53" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>38</v>
       </c>
@@ -6901,25 +7108,29 @@
         <v>11.4</v>
       </c>
       <c r="AD53" s="32">
+        <f t="shared" si="0"/>
+        <v>1.14E-2</v>
+      </c>
+      <c r="AE53">
         <v>0.19914999999999999</v>
       </c>
-      <c r="AE53" s="12">
+      <c r="AF53" s="12">
         <v>199.15</v>
       </c>
-      <c r="AF53" s="1">
+      <c r="AG53" s="1">
         <v>190</v>
       </c>
-      <c r="AG53">
+      <c r="AH53">
         <v>38</v>
       </c>
-      <c r="AH53">
+      <c r="AI53">
         <v>6.75</v>
       </c>
-      <c r="AI53" s="12">
+      <c r="AJ53" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="54" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>39</v>
       </c>
@@ -7008,25 +7219,29 @@
         <v>9.5</v>
       </c>
       <c r="AD54" s="32">
+        <f t="shared" si="0"/>
+        <v>9.4999999999999998E-3</v>
+      </c>
+      <c r="AE54">
         <v>0.18753999999999998</v>
       </c>
-      <c r="AE54" s="12">
+      <c r="AF54" s="12">
         <v>187.54</v>
       </c>
-      <c r="AF54" s="1">
+      <c r="AG54" s="1">
         <v>190</v>
       </c>
-      <c r="AG54">
+      <c r="AH54">
         <v>36.5</v>
       </c>
-      <c r="AH54">
+      <c r="AI54">
         <v>7.1</v>
       </c>
-      <c r="AI54" s="12">
+      <c r="AJ54" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="55" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>40</v>
       </c>
@@ -7115,25 +7330,29 @@
         <v>9.5</v>
       </c>
       <c r="AD55" s="32">
+        <f t="shared" si="0"/>
+        <v>9.4999999999999998E-3</v>
+      </c>
+      <c r="AE55">
         <v>0.18677000000000002</v>
       </c>
-      <c r="AE55" s="12">
+      <c r="AF55" s="12">
         <v>186.77</v>
       </c>
-      <c r="AF55" s="1">
+      <c r="AG55" s="1">
         <v>190</v>
       </c>
-      <c r="AG55">
+      <c r="AH55">
         <v>36.5</v>
       </c>
-      <c r="AH55">
+      <c r="AI55">
         <v>7.1</v>
       </c>
-      <c r="AI55" s="12">
+      <c r="AJ55" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="56" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:36" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>41</v>
       </c>
@@ -7222,25 +7441,29 @@
         <v>7.6</v>
       </c>
       <c r="AD56" s="32">
+        <f t="shared" si="0"/>
+        <v>7.6E-3</v>
+      </c>
+      <c r="AE56">
         <v>0.18778</v>
       </c>
-      <c r="AE56" s="12">
+      <c r="AF56" s="12">
         <v>187.78</v>
       </c>
-      <c r="AF56" s="1">
+      <c r="AG56" s="1">
         <v>190</v>
       </c>
-      <c r="AG56">
+      <c r="AH56">
         <v>35</v>
       </c>
-      <c r="AH56">
+      <c r="AI56">
         <v>7.45</v>
       </c>
-      <c r="AI56" s="12">
+      <c r="AJ56" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="57" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>36</v>
       </c>
@@ -7329,25 +7552,29 @@
         <v>0</v>
       </c>
       <c r="AD57" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE57" s="3">
         <v>0.18752000000000002</v>
       </c>
-      <c r="AE57" s="13">
+      <c r="AF57" s="13">
         <v>187.52</v>
       </c>
-      <c r="AF57" s="2">
+      <c r="AG57" s="2">
         <v>190</v>
       </c>
-      <c r="AG57" s="3">
+      <c r="AH57" s="3">
         <v>35</v>
       </c>
-      <c r="AH57" s="3">
+      <c r="AI57" s="3">
         <v>6.75</v>
       </c>
-      <c r="AI57" s="13">
+      <c r="AJ57" s="13">
         <v>40</v>
       </c>
     </row>
-    <row r="58" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>37</v>
       </c>
@@ -7436,25 +7663,29 @@
         <v>0</v>
       </c>
       <c r="AD58" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE58">
         <v>0.20965</v>
       </c>
-      <c r="AE58" s="12">
+      <c r="AF58" s="12">
         <v>209.65</v>
       </c>
-      <c r="AF58" s="1">
+      <c r="AG58" s="1">
         <v>190</v>
       </c>
-      <c r="AG58">
+      <c r="AH58">
         <v>35</v>
       </c>
-      <c r="AH58">
+      <c r="AI58">
         <v>7.45</v>
       </c>
-      <c r="AI58" s="12">
+      <c r="AJ58" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="59" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>38</v>
       </c>
@@ -7543,25 +7774,29 @@
         <v>0</v>
       </c>
       <c r="AD59" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE59">
         <v>0.19932</v>
       </c>
-      <c r="AE59" s="12">
+      <c r="AF59" s="12">
         <v>199.32</v>
       </c>
-      <c r="AF59" s="1">
+      <c r="AG59" s="1">
         <v>190</v>
       </c>
-      <c r="AG59">
+      <c r="AH59">
         <v>38</v>
       </c>
-      <c r="AH59">
+      <c r="AI59">
         <v>6.75</v>
       </c>
-      <c r="AI59" s="12">
+      <c r="AJ59" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="60" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>39</v>
       </c>
@@ -7650,25 +7885,29 @@
         <v>0</v>
       </c>
       <c r="AD60" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE60">
         <v>0.19721</v>
       </c>
-      <c r="AE60" s="12">
+      <c r="AF60" s="12">
         <v>197.21</v>
       </c>
-      <c r="AF60" s="1">
+      <c r="AG60" s="1">
         <v>190</v>
       </c>
-      <c r="AG60">
+      <c r="AH60">
         <v>36.5</v>
       </c>
-      <c r="AH60">
+      <c r="AI60">
         <v>7.1</v>
       </c>
-      <c r="AI60" s="12">
+      <c r="AJ60" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="61" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>40</v>
       </c>
@@ -7757,25 +7996,29 @@
         <v>0</v>
       </c>
       <c r="AD61" s="32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE61">
         <v>0.19469999999999998</v>
       </c>
-      <c r="AE61" s="12">
+      <c r="AF61" s="12">
         <v>194.7</v>
       </c>
-      <c r="AF61" s="1">
+      <c r="AG61" s="1">
         <v>190</v>
       </c>
-      <c r="AG61">
+      <c r="AH61">
         <v>36.5</v>
       </c>
-      <c r="AH61">
+      <c r="AI61">
         <v>7.1</v>
       </c>
-      <c r="AI61" s="12">
+      <c r="AJ61" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="62" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:36" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
         <v>41</v>
       </c>
@@ -7864,25 +8107,29 @@
         <v>0</v>
       </c>
       <c r="AD62" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE62" s="5">
         <v>0.19362000000000001</v>
       </c>
-      <c r="AE62" s="14">
+      <c r="AF62" s="14">
         <v>193.62</v>
       </c>
-      <c r="AF62" s="4">
+      <c r="AG62" s="4">
         <v>190</v>
       </c>
-      <c r="AG62" s="5">
+      <c r="AH62" s="5">
         <v>35</v>
       </c>
-      <c r="AH62" s="5">
+      <c r="AI62" s="5">
         <v>7.45</v>
       </c>
-      <c r="AI62" s="14">
+      <c r="AJ62" s="14">
         <v>40</v>
       </c>
     </row>
-    <row r="63" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>36</v>
       </c>
@@ -7971,25 +8218,29 @@
         <v>7.6</v>
       </c>
       <c r="AD63" s="32">
+        <f t="shared" si="0"/>
+        <v>7.6E-3</v>
+      </c>
+      <c r="AE63">
         <v>0.1923</v>
       </c>
-      <c r="AE63" s="12">
+      <c r="AF63" s="12">
         <v>192.3</v>
       </c>
-      <c r="AF63" s="1">
+      <c r="AG63" s="1">
         <v>190</v>
       </c>
-      <c r="AG63">
+      <c r="AH63">
         <v>35</v>
       </c>
-      <c r="AH63">
+      <c r="AI63">
         <v>6.75</v>
       </c>
-      <c r="AI63" s="12">
+      <c r="AJ63" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="64" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>37</v>
       </c>
@@ -8078,25 +8329,29 @@
         <v>11.4</v>
       </c>
       <c r="AD64" s="32">
+        <f t="shared" si="0"/>
+        <v>1.14E-2</v>
+      </c>
+      <c r="AE64">
         <v>0.21054</v>
       </c>
-      <c r="AE64" s="12">
+      <c r="AF64" s="12">
         <v>210.54</v>
       </c>
-      <c r="AF64" s="1">
+      <c r="AG64" s="1">
         <v>190</v>
       </c>
-      <c r="AG64">
+      <c r="AH64">
         <v>35</v>
       </c>
-      <c r="AH64">
+      <c r="AI64">
         <v>7.45</v>
       </c>
-      <c r="AI64" s="12">
+      <c r="AJ64" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="65" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>38</v>
       </c>
@@ -8185,25 +8440,29 @@
         <v>11.4</v>
       </c>
       <c r="AD65" s="32">
+        <f t="shared" si="0"/>
+        <v>1.14E-2</v>
+      </c>
+      <c r="AE65">
         <v>0.20788999999999999</v>
       </c>
-      <c r="AE65" s="12">
+      <c r="AF65" s="12">
         <v>207.89</v>
       </c>
-      <c r="AF65" s="1">
+      <c r="AG65" s="1">
         <v>190</v>
       </c>
-      <c r="AG65">
+      <c r="AH65">
         <v>38</v>
       </c>
-      <c r="AH65">
+      <c r="AI65">
         <v>6.75</v>
       </c>
-      <c r="AI65" s="12">
+      <c r="AJ65" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="66" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>39</v>
       </c>
@@ -8292,25 +8551,29 @@
         <v>9.5</v>
       </c>
       <c r="AD66" s="32">
+        <f t="shared" si="0"/>
+        <v>9.4999999999999998E-3</v>
+      </c>
+      <c r="AE66">
         <v>0.19563999999999998</v>
       </c>
-      <c r="AE66" s="12">
+      <c r="AF66" s="12">
         <v>195.64</v>
       </c>
-      <c r="AF66" s="1">
+      <c r="AG66" s="1">
         <v>190</v>
       </c>
-      <c r="AG66">
+      <c r="AH66">
         <v>36.5</v>
       </c>
-      <c r="AH66">
+      <c r="AI66">
         <v>7.1</v>
       </c>
-      <c r="AI66" s="12">
+      <c r="AJ66" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="67" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>40</v>
       </c>
@@ -8399,25 +8662,29 @@
         <v>9.5</v>
       </c>
       <c r="AD67" s="32">
+        <f t="shared" si="0"/>
+        <v>9.4999999999999998E-3</v>
+      </c>
+      <c r="AE67">
         <v>0.19494999999999998</v>
       </c>
-      <c r="AE67" s="12">
+      <c r="AF67" s="12">
         <v>194.95</v>
       </c>
-      <c r="AF67" s="1">
+      <c r="AG67" s="1">
         <v>190</v>
       </c>
-      <c r="AG67">
+      <c r="AH67">
         <v>36.5</v>
       </c>
-      <c r="AH67">
+      <c r="AI67">
         <v>7.1</v>
       </c>
-      <c r="AI67" s="12">
+      <c r="AJ67" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="68" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:36" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
         <v>41</v>
       </c>
@@ -8506,25 +8773,29 @@
         <v>7.6</v>
       </c>
       <c r="AD68" s="32">
+        <f t="shared" ref="AD68:AD92" si="1">AC68/1000</f>
+        <v>7.6E-3</v>
+      </c>
+      <c r="AE68">
         <v>0.19359000000000001</v>
       </c>
-      <c r="AE68" s="12">
+      <c r="AF68" s="12">
         <v>193.59</v>
       </c>
-      <c r="AF68" s="1">
+      <c r="AG68" s="1">
         <v>190</v>
       </c>
-      <c r="AG68">
+      <c r="AH68">
         <v>35</v>
       </c>
-      <c r="AH68">
+      <c r="AI68">
         <v>7.45</v>
       </c>
-      <c r="AI68" s="12">
+      <c r="AJ68" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="69" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>36</v>
       </c>
@@ -8613,25 +8884,29 @@
         <v>0</v>
       </c>
       <c r="AD69" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE69" s="3">
         <v>0.18947999999999998</v>
       </c>
-      <c r="AE69" s="13">
+      <c r="AF69" s="13">
         <v>189.48</v>
       </c>
-      <c r="AF69" s="2">
+      <c r="AG69" s="2">
         <v>190</v>
       </c>
-      <c r="AG69" s="3">
+      <c r="AH69" s="3">
         <v>35</v>
       </c>
-      <c r="AH69" s="3">
+      <c r="AI69" s="3">
         <v>6.75</v>
       </c>
-      <c r="AI69" s="13">
+      <c r="AJ69" s="13">
         <v>40</v>
       </c>
     </row>
-    <row r="70" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>37</v>
       </c>
@@ -8720,25 +8995,29 @@
         <v>0</v>
       </c>
       <c r="AD70" s="32">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE70">
         <v>0.22028999999999999</v>
       </c>
-      <c r="AE70" s="12">
+      <c r="AF70" s="12">
         <v>220.29</v>
       </c>
-      <c r="AF70" s="1">
+      <c r="AG70" s="1">
         <v>190</v>
       </c>
-      <c r="AG70">
+      <c r="AH70">
         <v>35</v>
       </c>
-      <c r="AH70">
+      <c r="AI70">
         <v>7.45</v>
       </c>
-      <c r="AI70" s="12">
+      <c r="AJ70" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="71" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>38</v>
       </c>
@@ -8827,25 +9106,29 @@
         <v>0</v>
       </c>
       <c r="AD71" s="32">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE71">
         <v>0.20648</v>
       </c>
-      <c r="AE71" s="12">
+      <c r="AF71" s="12">
         <v>206.48</v>
       </c>
-      <c r="AF71" s="1">
+      <c r="AG71" s="1">
         <v>190</v>
       </c>
-      <c r="AG71">
+      <c r="AH71">
         <v>38</v>
       </c>
-      <c r="AH71">
+      <c r="AI71">
         <v>6.75</v>
       </c>
-      <c r="AI71" s="12">
+      <c r="AJ71" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="72" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>39</v>
       </c>
@@ -8934,25 +9217,29 @@
         <v>0</v>
       </c>
       <c r="AD72" s="32">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE72">
         <v>0.20371</v>
       </c>
-      <c r="AE72" s="12">
+      <c r="AF72" s="12">
         <v>203.71</v>
       </c>
-      <c r="AF72" s="1">
+      <c r="AG72" s="1">
         <v>190</v>
       </c>
-      <c r="AG72">
+      <c r="AH72">
         <v>36.5</v>
       </c>
-      <c r="AH72">
+      <c r="AI72">
         <v>7.1</v>
       </c>
-      <c r="AI72" s="12">
+      <c r="AJ72" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="73" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>40</v>
       </c>
@@ -9041,25 +9328,29 @@
         <v>0</v>
       </c>
       <c r="AD73" s="32">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE73">
         <v>0.20305000000000001</v>
       </c>
-      <c r="AE73" s="12">
+      <c r="AF73" s="12">
         <v>203.05</v>
       </c>
-      <c r="AF73" s="1">
+      <c r="AG73" s="1">
         <v>190</v>
       </c>
-      <c r="AG73">
+      <c r="AH73">
         <v>36.5</v>
       </c>
-      <c r="AH73">
+      <c r="AI73">
         <v>7.1</v>
       </c>
-      <c r="AI73" s="12">
+      <c r="AJ73" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="74" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:36" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
         <v>41</v>
       </c>
@@ -9148,25 +9439,29 @@
         <v>0</v>
       </c>
       <c r="AD74" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE74" s="5">
         <v>0.19938999999999998</v>
       </c>
-      <c r="AE74" s="14">
+      <c r="AF74" s="14">
         <v>199.39</v>
       </c>
-      <c r="AF74" s="4">
+      <c r="AG74" s="4">
         <v>190</v>
       </c>
-      <c r="AG74" s="5">
+      <c r="AH74" s="5">
         <v>35</v>
       </c>
-      <c r="AH74" s="5">
+      <c r="AI74" s="5">
         <v>7.45</v>
       </c>
-      <c r="AI74" s="14">
+      <c r="AJ74" s="14">
         <v>40</v>
       </c>
     </row>
-    <row r="75" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>36</v>
       </c>
@@ -9255,25 +9550,29 @@
         <v>7.6</v>
       </c>
       <c r="AD75" s="32">
+        <f t="shared" si="1"/>
+        <v>7.6E-3</v>
+      </c>
+      <c r="AE75">
         <v>0.19427</v>
       </c>
-      <c r="AE75" s="12">
+      <c r="AF75" s="12">
         <v>194.27</v>
       </c>
-      <c r="AF75" s="1">
+      <c r="AG75" s="1">
         <v>190</v>
       </c>
-      <c r="AG75">
+      <c r="AH75">
         <v>35</v>
       </c>
-      <c r="AH75">
+      <c r="AI75">
         <v>6.75</v>
       </c>
-      <c r="AI75" s="12">
+      <c r="AJ75" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="76" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>37</v>
       </c>
@@ -9362,25 +9661,29 @@
         <v>11.4</v>
       </c>
       <c r="AD76" s="32">
+        <f t="shared" si="1"/>
+        <v>1.14E-2</v>
+      </c>
+      <c r="AE76">
         <v>0.21881</v>
       </c>
-      <c r="AE76" s="12">
+      <c r="AF76" s="12">
         <v>218.81</v>
       </c>
-      <c r="AF76" s="1">
+      <c r="AG76" s="1">
         <v>190</v>
       </c>
-      <c r="AG76">
+      <c r="AH76">
         <v>35</v>
       </c>
-      <c r="AH76">
+      <c r="AI76">
         <v>7.45</v>
       </c>
-      <c r="AI76" s="12">
+      <c r="AJ76" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="77" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>38</v>
       </c>
@@ -9469,25 +9772,29 @@
         <v>11.4</v>
       </c>
       <c r="AD77" s="32">
+        <f t="shared" si="1"/>
+        <v>1.14E-2</v>
+      </c>
+      <c r="AE77">
         <v>0.21505000000000002</v>
       </c>
-      <c r="AE77" s="12">
+      <c r="AF77" s="12">
         <v>215.05</v>
       </c>
-      <c r="AF77" s="1">
+      <c r="AG77" s="1">
         <v>190</v>
       </c>
-      <c r="AG77">
+      <c r="AH77">
         <v>38</v>
       </c>
-      <c r="AH77">
+      <c r="AI77">
         <v>6.75</v>
       </c>
-      <c r="AI77" s="12">
+      <c r="AJ77" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="78" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>39</v>
       </c>
@@ -9576,25 +9883,29 @@
         <v>9.5</v>
       </c>
       <c r="AD78" s="32">
+        <f t="shared" si="1"/>
+        <v>9.4999999999999998E-3</v>
+      </c>
+      <c r="AE78">
         <v>0.20225000000000001</v>
       </c>
-      <c r="AE78" s="12">
+      <c r="AF78" s="12">
         <v>202.25</v>
       </c>
-      <c r="AF78" s="1">
+      <c r="AG78" s="1">
         <v>190</v>
       </c>
-      <c r="AG78">
+      <c r="AH78">
         <v>36.5</v>
       </c>
-      <c r="AH78">
+      <c r="AI78">
         <v>7.1</v>
       </c>
-      <c r="AI78" s="12">
+      <c r="AJ78" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="79" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>40</v>
       </c>
@@ -9683,25 +9994,29 @@
         <v>9.5</v>
       </c>
       <c r="AD79" s="32">
+        <f t="shared" si="1"/>
+        <v>9.4999999999999998E-3</v>
+      </c>
+      <c r="AE79">
         <v>0.2016</v>
       </c>
-      <c r="AE79" s="12">
+      <c r="AF79" s="12">
         <v>201.6</v>
       </c>
-      <c r="AF79" s="1">
+      <c r="AG79" s="1">
         <v>190</v>
       </c>
-      <c r="AG79">
+      <c r="AH79">
         <v>36.5</v>
       </c>
-      <c r="AH79">
+      <c r="AI79">
         <v>7.1</v>
       </c>
-      <c r="AI79" s="12">
+      <c r="AJ79" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="80" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:36" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
         <v>41</v>
       </c>
@@ -9790,25 +10105,29 @@
         <v>7.6</v>
       </c>
       <c r="AD80" s="32">
+        <f t="shared" si="1"/>
+        <v>7.6E-3</v>
+      </c>
+      <c r="AE80">
         <v>0.19769999999999999</v>
       </c>
-      <c r="AE80" s="12">
+      <c r="AF80" s="12">
         <v>197.7</v>
       </c>
-      <c r="AF80" s="1">
+      <c r="AG80" s="1">
         <v>190</v>
       </c>
-      <c r="AG80">
+      <c r="AH80">
         <v>35</v>
       </c>
-      <c r="AH80">
+      <c r="AI80">
         <v>7.45</v>
       </c>
-      <c r="AI80" s="12">
+      <c r="AJ80" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="81" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>36</v>
       </c>
@@ -9897,25 +10216,29 @@
         <v>0</v>
       </c>
       <c r="AD81" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE81" s="3">
         <v>0.19272</v>
       </c>
-      <c r="AE81" s="13">
+      <c r="AF81" s="13">
         <v>192.72</v>
       </c>
-      <c r="AF81" s="2">
+      <c r="AG81" s="2">
         <v>190</v>
       </c>
-      <c r="AG81" s="3">
+      <c r="AH81" s="3">
         <v>35</v>
       </c>
-      <c r="AH81" s="3">
+      <c r="AI81" s="3">
         <v>6.75</v>
       </c>
-      <c r="AI81" s="13">
+      <c r="AJ81" s="13">
         <v>40</v>
       </c>
     </row>
-    <row r="82" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>37</v>
       </c>
@@ -10004,25 +10327,29 @@
         <v>0</v>
       </c>
       <c r="AD82" s="32">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE82">
         <v>0.22853999999999999</v>
       </c>
-      <c r="AE82" s="12">
+      <c r="AF82" s="12">
         <v>228.54</v>
       </c>
-      <c r="AF82" s="1">
+      <c r="AG82" s="1">
         <v>190</v>
       </c>
-      <c r="AG82">
+      <c r="AH82">
         <v>35</v>
       </c>
-      <c r="AH82">
+      <c r="AI82">
         <v>7.45</v>
       </c>
-      <c r="AI82" s="12">
+      <c r="AJ82" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="83" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>38</v>
       </c>
@@ -10111,25 +10438,29 @@
         <v>0</v>
       </c>
       <c r="AD83" s="32">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE83">
         <v>0.21383000000000002</v>
       </c>
-      <c r="AE83" s="12">
+      <c r="AF83" s="12">
         <v>213.83</v>
       </c>
-      <c r="AF83" s="1">
+      <c r="AG83" s="1">
         <v>190</v>
       </c>
-      <c r="AG83">
+      <c r="AH83">
         <v>38</v>
       </c>
-      <c r="AH83">
+      <c r="AI83">
         <v>6.75</v>
       </c>
-      <c r="AI83" s="12">
+      <c r="AJ83" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="84" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>39</v>
       </c>
@@ -10218,25 +10549,29 @@
         <v>0</v>
       </c>
       <c r="AD84" s="32">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE84">
         <v>0.21038999999999999</v>
       </c>
-      <c r="AE84" s="12">
+      <c r="AF84" s="12">
         <v>210.39</v>
       </c>
-      <c r="AF84" s="1">
+      <c r="AG84" s="1">
         <v>190</v>
       </c>
-      <c r="AG84">
+      <c r="AH84">
         <v>36.5</v>
       </c>
-      <c r="AH84">
+      <c r="AI84">
         <v>7.1</v>
       </c>
-      <c r="AI84" s="12">
+      <c r="AJ84" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="85" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>40</v>
       </c>
@@ -10325,25 +10660,29 @@
         <v>0</v>
       </c>
       <c r="AD85" s="32">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE85">
         <v>0.20957000000000001</v>
       </c>
-      <c r="AE85" s="12">
+      <c r="AF85" s="12">
         <v>209.57</v>
       </c>
-      <c r="AF85" s="1">
+      <c r="AG85" s="1">
         <v>190</v>
       </c>
-      <c r="AG85">
+      <c r="AH85">
         <v>36.5</v>
       </c>
-      <c r="AH85">
+      <c r="AI85">
         <v>7.1</v>
       </c>
-      <c r="AI85" s="12">
+      <c r="AJ85" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="86" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:36" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A86" s="4" t="s">
         <v>41</v>
       </c>
@@ -10432,25 +10771,29 @@
         <v>0</v>
       </c>
       <c r="AD86" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE86" s="5">
         <v>0.20361000000000001</v>
       </c>
-      <c r="AE86" s="14">
+      <c r="AF86" s="14">
         <v>203.61</v>
       </c>
-      <c r="AF86" s="4">
+      <c r="AG86" s="4">
         <v>190</v>
       </c>
-      <c r="AG86" s="5">
+      <c r="AH86" s="5">
         <v>35</v>
       </c>
-      <c r="AH86" s="5">
+      <c r="AI86" s="5">
         <v>7.45</v>
       </c>
-      <c r="AI86" s="14">
+      <c r="AJ86" s="14">
         <v>40</v>
       </c>
     </row>
-    <row r="87" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
         <v>36</v>
       </c>
@@ -10539,25 +10882,29 @@
         <v>0</v>
       </c>
       <c r="AD87" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE87" s="3">
         <v>0.18809999999999999</v>
       </c>
-      <c r="AE87" s="13">
+      <c r="AF87" s="13">
         <v>188.1</v>
       </c>
-      <c r="AF87" s="2">
+      <c r="AG87" s="2">
         <v>190</v>
       </c>
-      <c r="AG87" s="3">
+      <c r="AH87" s="3">
         <v>35</v>
       </c>
-      <c r="AH87" s="3">
+      <c r="AI87" s="3">
         <v>6.75</v>
       </c>
-      <c r="AI87" s="13">
+      <c r="AJ87" s="13">
         <v>40</v>
       </c>
     </row>
-    <row r="88" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>37</v>
       </c>
@@ -10646,25 +10993,29 @@
         <v>0</v>
       </c>
       <c r="AD88" s="32">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE88">
         <v>0.22525999999999999</v>
       </c>
-      <c r="AE88" s="12">
+      <c r="AF88" s="12">
         <v>225.26</v>
       </c>
-      <c r="AF88" s="1">
+      <c r="AG88" s="1">
         <v>190</v>
       </c>
-      <c r="AG88">
+      <c r="AH88">
         <v>35</v>
       </c>
-      <c r="AH88">
+      <c r="AI88">
         <v>7.45</v>
       </c>
-      <c r="AI88" s="12">
+      <c r="AJ88" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="89" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>38</v>
       </c>
@@ -10753,25 +11104,29 @@
         <v>0</v>
       </c>
       <c r="AD89" s="32">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE89">
         <v>0.20921000000000001</v>
       </c>
-      <c r="AE89" s="12">
+      <c r="AF89" s="12">
         <v>209.21</v>
       </c>
-      <c r="AF89" s="1">
+      <c r="AG89" s="1">
         <v>190</v>
       </c>
-      <c r="AG89">
+      <c r="AH89">
         <v>38</v>
       </c>
-      <c r="AH89">
+      <c r="AI89">
         <v>6.75</v>
       </c>
-      <c r="AI89" s="12">
+      <c r="AJ89" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="90" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>39</v>
       </c>
@@ -10860,25 +11215,29 @@
         <v>0</v>
       </c>
       <c r="AD90" s="32">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE90">
         <v>0.20710000000000001</v>
       </c>
-      <c r="AE90" s="12">
+      <c r="AF90" s="12">
         <v>207.1</v>
       </c>
-      <c r="AF90" s="1">
+      <c r="AG90" s="1">
         <v>190</v>
       </c>
-      <c r="AG90">
+      <c r="AH90">
         <v>36.5</v>
       </c>
-      <c r="AH90">
+      <c r="AI90">
         <v>7.1</v>
       </c>
-      <c r="AI90" s="12">
+      <c r="AJ90" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="91" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>40</v>
       </c>
@@ -10967,25 +11326,29 @@
         <v>0</v>
       </c>
       <c r="AD91" s="32">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE91">
         <v>0.20627000000000001</v>
       </c>
-      <c r="AE91" s="12">
+      <c r="AF91" s="12">
         <v>206.27</v>
       </c>
-      <c r="AF91" s="1">
+      <c r="AG91" s="1">
         <v>190</v>
       </c>
-      <c r="AG91">
+      <c r="AH91">
         <v>36.5</v>
       </c>
-      <c r="AH91">
+      <c r="AI91">
         <v>7.1</v>
       </c>
-      <c r="AI91" s="12">
+      <c r="AJ91" s="12">
         <v>40</v>
       </c>
     </row>
-    <row r="92" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:36" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A92" s="4" t="s">
         <v>41</v>
       </c>
@@ -11074,35 +11437,39 @@
         <v>0</v>
       </c>
       <c r="AD92" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE92" s="5">
         <v>0.20033999999999999</v>
       </c>
-      <c r="AE92" s="14">
+      <c r="AF92" s="14">
         <v>200.34</v>
       </c>
-      <c r="AF92" s="4">
+      <c r="AG92" s="4">
         <v>190</v>
       </c>
-      <c r="AG92" s="5">
+      <c r="AH92" s="5">
         <v>35</v>
       </c>
-      <c r="AH92" s="5">
+      <c r="AI92" s="5">
         <v>7.45</v>
       </c>
-      <c r="AI92" s="14">
+      <c r="AJ92" s="14">
         <v>40</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AI92" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:AI92">
+  <autoFilter ref="A2:AJ92" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:AJ92">
       <sortCondition ref="E2:E92"/>
     </sortState>
   </autoFilter>
   <mergeCells count="4">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="G1:AB1"/>
-    <mergeCell ref="AF1:AI1"/>
-    <mergeCell ref="AC1:AE1"/>
+    <mergeCell ref="AG1:AJ1"/>
+    <mergeCell ref="AC1:AF1"/>
   </mergeCells>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11113,9 +11480,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{964DBE78-A1C2-42B9-8531-C1C4562D2F57}">
   <dimension ref="A1:F46"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>42</v>
       </c>
@@ -11126,7 +11493,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -11141,7 +11508,7 @@
         <v>70.175349999999995</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>0</v>
       </c>
@@ -11156,7 +11523,7 @@
         <v>70.441850000000002</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>0</v>
       </c>
@@ -11171,7 +11538,7 @@
         <v>67.848200000000006</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -11186,7 +11553,7 @@
         <v>99.879050000000007</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1</v>
       </c>
@@ -11201,7 +11568,7 @@
         <v>199.21946666666668</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1</v>
       </c>
@@ -11216,7 +11583,7 @@
         <v>333.67943333333329</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2</v>
       </c>
@@ -11231,7 +11598,7 @@
         <v>581.69326666666666</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2</v>
       </c>
@@ -11246,7 +11613,7 @@
         <v>753.39584533333345</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2</v>
       </c>
@@ -11261,7 +11628,7 @@
         <v>1268.3525340000001</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>3</v>
       </c>
@@ -11276,7 +11643,7 @@
         <v>1592.0958713333334</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>3</v>
       </c>
@@ -11291,7 +11658,7 @@
         <v>2151.9790066666669</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>3</v>
       </c>
@@ -11306,7 +11673,7 @@
         <v>2589.1378500000001</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>4</v>
       </c>
@@ -11321,7 +11688,7 @@
         <v>2951.6538500000006</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>4</v>
       </c>
@@ -11336,7 +11703,7 @@
         <v>3102.8715999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>4</v>
       </c>
@@ -11351,7 +11718,7 @@
         <v>3544.1503000000007</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>5</v>
       </c>
@@ -11359,7 +11726,7 @@
         <v>408.03620000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>5</v>
       </c>
@@ -11367,7 +11734,7 @@
         <v>175.25470000000001</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>5</v>
       </c>
@@ -11375,7 +11742,7 @@
         <v>417.74740000000003</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>6</v>
       </c>
@@ -11383,7 +11750,7 @@
         <v>693.36239999999998</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>6</v>
       </c>
@@ -11391,7 +11758,7 @@
         <v>306.12569999999999</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>6</v>
       </c>
@@ -11399,7 +11766,7 @@
         <v>745.59169999999995</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>7</v>
       </c>
@@ -11407,7 +11774,7 @@
         <v>823.29169999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>7</v>
       </c>
@@ -11415,7 +11782,7 @@
         <v>372.73790000000002</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>7</v>
       </c>
@@ -11423,7 +11790,7 @@
         <v>916.29520000000002</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>8</v>
       </c>
@@ -11431,7 +11798,7 @@
         <v>1337.0650000000001</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>8</v>
       </c>
@@ -11439,7 +11806,7 @@
         <v>671.00360000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>8</v>
       </c>
@@ -11447,7 +11814,7 @@
         <v>1548.06</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>9</v>
       </c>
@@ -11455,7 +11822,7 @@
         <v>1767.66</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>9</v>
       </c>
@@ -11463,7 +11830,7 @@
         <v>876.37519999999995</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>9</v>
       </c>
@@ -11471,7 +11838,7 @@
         <v>1819.7850000000001</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>10</v>
       </c>
@@ -11479,7 +11846,7 @@
         <v>2326.5450000000001</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>10</v>
       </c>
@@ -11487,7 +11854,7 @@
         <v>1296.181</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>10</v>
       </c>
@@ -11495,7 +11862,7 @@
         <v>2410.86</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>11</v>
       </c>
@@ -11503,7 +11870,7 @@
         <v>2798.2049999999999</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>11</v>
       </c>
@@ -11511,7 +11878,7 @@
         <v>1673.64</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>11</v>
       </c>
@@ -11519,7 +11886,7 @@
         <v>2787.42</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>12</v>
       </c>
@@ -11527,7 +11894,7 @@
         <v>3099.57</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>12</v>
       </c>
@@ -11535,7 +11902,7 @@
         <v>2063.79</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>12</v>
       </c>
@@ -11543,7 +11910,7 @@
         <v>3112.3049999999998</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>13</v>
       </c>
@@ -11551,7 +11918,7 @@
         <v>3206.2649999999999</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>13</v>
       </c>
@@ -11559,7 +11926,7 @@
         <v>2248.2750000000001</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>13</v>
       </c>
@@ -11567,7 +11934,7 @@
         <v>3245.1</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>14</v>
       </c>
@@ -11575,7 +11942,7 @@
         <v>3758.5650000000001</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>14</v>
       </c>
@@ -11583,7 +11950,7 @@
         <v>2667.4050000000002</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>14</v>
       </c>
@@ -11598,33 +11965,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34d8c884-fe7e-4d4f-a833-b92a2823f74b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <SharedWithUsers xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B75172DAFC2BB6479729CB287362C7E3" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0fc11b0946794a47057850b4f6c92dd7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34d8c884-fe7e-4d4f-a833-b92a2823f74b" xmlns:ns3="a198008e-c7f6-4ed0-9865-26ace3c97b59" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fb90ec7fe59ed1d44226abab88cd233b" ns2:_="" ns3:_="">
     <xsd:import namespace="34d8c884-fe7e-4d4f-a833-b92a2823f74b"/>
@@ -11847,10 +12187,48 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34d8c884-fe7e-4d4f-a833-b92a2823f74b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <SharedWithUsers xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FA2C79D-5C43-4F8C-8CB2-6CBFC4591548}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F43DC28-AE43-4EFF-8739-4E0C557B415B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="34d8c884-fe7e-4d4f-a833-b92a2823f74b"/>
+    <ds:schemaRef ds:uri="a198008e-c7f6-4ed0-9865-26ace3c97b59"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11867,20 +12245,15 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F43DC28-AE43-4EFF-8739-4E0C557B415B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FA2C79D-5C43-4F8C-8CB2-6CBFC4591548}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="34d8c884-fe7e-4d4f-a833-b92a2823f74b"/>
-    <ds:schemaRef ds:uri="a198008e-c7f6-4ed0-9865-26ace3c97b59"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{bea66b2b-af80-48b6-873b-d341d3035cfa}" enabled="1" method="Standard" siteId="{63982aff-fb6c-4c22-973b-70e4acfb63e6}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>